<commit_message>
DASH / WEB SERVICE / SIM DEVELOPMENT
</commit_message>
<xml_diff>
--- a/mx5.xlsx
+++ b/mx5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aiformaneuver-my.sharepoint.us/personal/rob_kuelbs_shield_ai/Documents/Documents/Miata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{88A26781-0A8E-4E49-9E21-C4F39EEBF44C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{88A26781-0A8E-4E49-9E21-C4F39EEBF44C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A64B57F-8BB1-4844-A5CD-596278D4E2DC}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="17520" activeTab="5" xr2:uid="{5CB7ED78-F18E-4FF4-B78C-6300A5C08EC5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{5CB7ED78-F18E-4FF4-B78C-6300A5C08EC5}"/>
   </bookViews>
   <sheets>
     <sheet name="MEL" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1054" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1058" uniqueCount="452">
   <si>
     <t>LIGHTING</t>
   </si>
@@ -1325,9 +1325,6 @@
     <t>HIGH_BEAM_N</t>
   </si>
   <si>
-    <t>HEADLIGHTS_N</t>
-  </si>
-  <si>
     <t>ACC_OUT_N</t>
   </si>
   <si>
@@ -1401,6 +1398,15 @@
   </si>
   <si>
     <t>SHOCK POTS</t>
+  </si>
+  <si>
+    <t>FUEL LEVEL SENSOR</t>
+  </si>
+  <si>
+    <t>FUEL_LEVEL</t>
+  </si>
+  <si>
+    <t>LOW_BEAM_N</t>
   </si>
 </sst>
 </file>
@@ -3943,7 +3949,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{383E71EB-5C1B-4B6B-BB19-94D0D800893B}">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="23.7109375" customWidth="1"/>
@@ -3981,213 +3987,234 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>298</v>
+        <v>253</v>
       </c>
       <c r="C2" t="s">
-        <v>296</v>
+        <v>248</v>
       </c>
       <c r="D2" t="s">
-        <v>297</v>
+        <v>257</v>
       </c>
       <c r="E2" t="s">
-        <v>404</v>
+        <v>388</v>
+      </c>
+      <c r="F2" t="s">
+        <v>302</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>299</v>
+        <v>254</v>
       </c>
       <c r="C3" t="s">
-        <v>296</v>
+        <v>248</v>
       </c>
       <c r="D3" t="s">
-        <v>297</v>
+        <v>257</v>
       </c>
       <c r="E3" t="s">
-        <v>405</v>
+        <v>391</v>
+      </c>
+      <c r="F3" t="s">
+        <v>302</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>362</v>
+        <v>255</v>
       </c>
       <c r="C4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D4" t="s">
-        <v>93</v>
+        <v>257</v>
+      </c>
+      <c r="E4" t="s">
+        <v>389</v>
       </c>
       <c r="F4" t="s">
-        <v>408</v>
-      </c>
-      <c r="G4" t="s">
-        <v>363</v>
+        <v>302</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>406</v>
+        <v>256</v>
       </c>
       <c r="C5" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D5" t="s">
-        <v>93</v>
+        <v>257</v>
       </c>
       <c r="E5" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="F5" t="s">
-        <v>407</v>
+        <v>302</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C6" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D6" t="s">
-        <v>93</v>
+        <v>257</v>
       </c>
       <c r="E6" t="s">
-        <v>396</v>
+        <v>412</v>
       </c>
       <c r="F6" t="s">
-        <v>407</v>
+        <v>300</v>
       </c>
       <c r="G6" t="s">
-        <v>293</v>
+        <v>307</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>251</v>
+        <v>303</v>
       </c>
       <c r="C7" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D7" t="s">
-        <v>93</v>
+        <v>257</v>
       </c>
       <c r="E7" t="s">
-        <v>393</v>
+        <v>413</v>
+      </c>
+      <c r="F7" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="C8" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D8" t="s">
-        <v>93</v>
+        <v>257</v>
       </c>
       <c r="E8" t="s">
-        <v>403</v>
-      </c>
-      <c r="G8" t="s">
-        <v>314</v>
+        <v>414</v>
+      </c>
+      <c r="F8" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>397</v>
+        <v>313</v>
       </c>
       <c r="C9" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D9" t="s">
-        <v>93</v>
+        <v>257</v>
       </c>
       <c r="E9" t="s">
-        <v>398</v>
+        <v>415</v>
+      </c>
+      <c r="F9" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>290</v>
+        <v>19</v>
       </c>
       <c r="C10" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D10" t="s">
         <v>257</v>
       </c>
       <c r="E10" t="s">
-        <v>394</v>
-      </c>
-      <c r="G10" t="s">
-        <v>292</v>
+        <v>416</v>
+      </c>
+      <c r="F10" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>291</v>
+        <v>399</v>
       </c>
       <c r="C11" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D11" t="s">
         <v>257</v>
       </c>
       <c r="E11" t="s">
-        <v>395</v>
-      </c>
-      <c r="G11" t="s">
-        <v>292</v>
+        <v>417</v>
+      </c>
+      <c r="F11" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>323</v>
+        <v>402</v>
       </c>
       <c r="C12" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D12" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="E12" t="s">
-        <v>386</v>
-      </c>
-      <c r="G12" t="s">
-        <v>324</v>
+        <v>418</v>
+      </c>
+      <c r="F12" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>384</v>
+        <v>362</v>
       </c>
       <c r="C13" t="s">
         <v>247</v>
       </c>
       <c r="D13" t="s">
-        <v>257</v>
-      </c>
-      <c r="E13" t="s">
-        <v>400</v>
+        <v>93</v>
+      </c>
+      <c r="F13" t="s">
+        <v>408</v>
+      </c>
+      <c r="G13" t="s">
+        <v>363</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>365</v>
+        <v>409</v>
       </c>
       <c r="C14" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D14" t="s">
         <v>257</v>
       </c>
       <c r="E14" t="s">
-        <v>401</v>
+        <v>411</v>
+      </c>
+      <c r="F14" t="s">
+        <v>304</v>
+      </c>
+      <c r="G14" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C15" t="s">
         <v>248</v>
@@ -4196,7 +4223,7 @@
         <v>257</v>
       </c>
       <c r="E15" t="s">
-        <v>411</v>
+        <v>390</v>
       </c>
       <c r="F15" t="s">
         <v>304</v>
@@ -4207,7 +4234,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>410</v>
+        <v>419</v>
       </c>
       <c r="C16" t="s">
         <v>248</v>
@@ -4216,7 +4243,7 @@
         <v>257</v>
       </c>
       <c r="E16" t="s">
-        <v>390</v>
+        <v>421</v>
       </c>
       <c r="F16" t="s">
         <v>304</v>
@@ -4227,7 +4254,7 @@
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>253</v>
+        <v>420</v>
       </c>
       <c r="C17" t="s">
         <v>248</v>
@@ -4236,15 +4263,18 @@
         <v>257</v>
       </c>
       <c r="E17" t="s">
-        <v>388</v>
+        <v>422</v>
       </c>
       <c r="F17" t="s">
-        <v>302</v>
+        <v>304</v>
+      </c>
+      <c r="G17" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>254</v>
+        <v>316</v>
       </c>
       <c r="C18" t="s">
         <v>248</v>
@@ -4253,15 +4283,18 @@
         <v>257</v>
       </c>
       <c r="E18" t="s">
-        <v>391</v>
+        <v>423</v>
       </c>
       <c r="F18" t="s">
-        <v>302</v>
+        <v>304</v>
+      </c>
+      <c r="G18" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>255</v>
+        <v>317</v>
       </c>
       <c r="C19" t="s">
         <v>248</v>
@@ -4270,15 +4303,18 @@
         <v>257</v>
       </c>
       <c r="E19" t="s">
-        <v>389</v>
+        <v>451</v>
       </c>
       <c r="F19" t="s">
-        <v>302</v>
+        <v>304</v>
+      </c>
+      <c r="G19" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
-        <v>256</v>
+        <v>306</v>
       </c>
       <c r="C20" t="s">
         <v>248</v>
@@ -4287,15 +4323,18 @@
         <v>257</v>
       </c>
       <c r="E20" t="s">
-        <v>392</v>
+        <v>424</v>
       </c>
       <c r="F20" t="s">
-        <v>302</v>
+        <v>304</v>
+      </c>
+      <c r="G20" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>295</v>
+        <v>425</v>
       </c>
       <c r="C21" t="s">
         <v>248</v>
@@ -4304,278 +4343,259 @@
         <v>257</v>
       </c>
       <c r="E21" t="s">
-        <v>412</v>
+        <v>426</v>
       </c>
       <c r="F21" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G21" t="s">
-        <v>307</v>
+        <v>318</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>303</v>
+        <v>427</v>
       </c>
       <c r="C22" t="s">
         <v>248</v>
       </c>
       <c r="D22" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="E22" t="s">
-        <v>413</v>
+        <v>428</v>
       </c>
       <c r="F22" t="s">
-        <v>300</v>
+        <v>304</v>
+      </c>
+      <c r="G22" t="s">
+        <v>427</v>
       </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>312</v>
+        <v>406</v>
       </c>
       <c r="C23" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D23" t="s">
-        <v>257</v>
+        <v>93</v>
       </c>
       <c r="E23" t="s">
-        <v>414</v>
+        <v>387</v>
       </c>
       <c r="F23" t="s">
-        <v>300</v>
+        <v>407</v>
       </c>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>313</v>
+        <v>294</v>
       </c>
       <c r="C24" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D24" t="s">
-        <v>257</v>
+        <v>93</v>
       </c>
       <c r="E24" t="s">
-        <v>415</v>
+        <v>396</v>
       </c>
       <c r="F24" t="s">
-        <v>300</v>
+        <v>407</v>
+      </c>
+      <c r="G24" t="s">
+        <v>293</v>
       </c>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>19</v>
+        <v>298</v>
       </c>
       <c r="C25" t="s">
-        <v>248</v>
+        <v>296</v>
       </c>
       <c r="D25" t="s">
-        <v>257</v>
+        <v>297</v>
       </c>
       <c r="E25" t="s">
-        <v>416</v>
-      </c>
-      <c r="F25" t="s">
-        <v>300</v>
+        <v>404</v>
       </c>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>399</v>
+        <v>299</v>
       </c>
       <c r="C26" t="s">
-        <v>248</v>
+        <v>296</v>
       </c>
       <c r="D26" t="s">
-        <v>257</v>
+        <v>297</v>
       </c>
       <c r="E26" t="s">
-        <v>417</v>
-      </c>
-      <c r="F26" t="s">
-        <v>300</v>
+        <v>405</v>
       </c>
     </row>
     <row r="27" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>402</v>
+        <v>251</v>
       </c>
       <c r="C27" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D27" t="s">
-        <v>249</v>
+        <v>93</v>
       </c>
       <c r="E27" t="s">
-        <v>418</v>
-      </c>
-      <c r="F27" t="s">
-        <v>300</v>
+        <v>393</v>
       </c>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>419</v>
+        <v>315</v>
       </c>
       <c r="C28" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D28" t="s">
-        <v>257</v>
+        <v>93</v>
       </c>
       <c r="E28" t="s">
-        <v>421</v>
-      </c>
-      <c r="F28" t="s">
-        <v>304</v>
+        <v>403</v>
       </c>
       <c r="G28" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
-        <v>420</v>
+        <v>397</v>
       </c>
       <c r="C29" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D29" t="s">
-        <v>257</v>
+        <v>93</v>
       </c>
       <c r="E29" t="s">
-        <v>422</v>
-      </c>
-      <c r="F29" t="s">
-        <v>304</v>
-      </c>
-      <c r="G29" t="s">
-        <v>318</v>
+        <v>398</v>
       </c>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
-        <v>316</v>
+        <v>290</v>
       </c>
       <c r="C30" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D30" t="s">
         <v>257</v>
       </c>
       <c r="E30" t="s">
-        <v>423</v>
-      </c>
-      <c r="F30" t="s">
-        <v>304</v>
+        <v>394</v>
       </c>
       <c r="G30" t="s">
-        <v>318</v>
+        <v>292</v>
       </c>
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
-        <v>317</v>
+        <v>291</v>
       </c>
       <c r="C31" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D31" t="s">
         <v>257</v>
       </c>
       <c r="E31" t="s">
-        <v>424</v>
-      </c>
-      <c r="F31" t="s">
-        <v>304</v>
+        <v>395</v>
       </c>
       <c r="G31" t="s">
-        <v>318</v>
+        <v>292</v>
       </c>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>306</v>
+        <v>323</v>
       </c>
       <c r="C32" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D32" t="s">
         <v>257</v>
       </c>
       <c r="E32" t="s">
-        <v>425</v>
-      </c>
-      <c r="F32" t="s">
-        <v>304</v>
+        <v>386</v>
       </c>
       <c r="G32" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
-        <v>250</v>
+        <v>384</v>
       </c>
       <c r="C33" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D33" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="E33" t="s">
-        <v>369</v>
-      </c>
-      <c r="G33" t="s">
-        <v>252</v>
+        <v>400</v>
       </c>
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
-        <v>426</v>
+        <v>365</v>
       </c>
       <c r="C34" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D34" t="s">
         <v>257</v>
       </c>
       <c r="E34" t="s">
-        <v>427</v>
-      </c>
-      <c r="F34" t="s">
-        <v>304</v>
-      </c>
-      <c r="G34" t="s">
-        <v>318</v>
+        <v>401</v>
       </c>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
-        <v>428</v>
+        <v>250</v>
       </c>
       <c r="C35" t="s">
         <v>248</v>
       </c>
       <c r="D35" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="E35" t="s">
-        <v>429</v>
-      </c>
-      <c r="F35" t="s">
-        <v>304</v>
+        <v>369</v>
       </c>
       <c r="G35" t="s">
-        <v>428</v>
+        <v>252</v>
+      </c>
+    </row>
+    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B36" t="s">
+        <v>449</v>
+      </c>
+      <c r="C36" t="s">
+        <v>247</v>
+      </c>
+      <c r="D36" t="s">
+        <v>93</v>
+      </c>
+      <c r="E36" t="s">
+        <v>450</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="B1:G1" xr:uid="{383E71EB-5C1B-4B6B-BB19-94D0D800893B}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:G32">
-      <sortCondition ref="C1"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:G36">
+      <sortCondition ref="F1"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4834,22 +4854,22 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
@@ -4864,7 +4884,7 @@
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
   </sheetData>
@@ -6988,13 +7008,13 @@
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C51" t="s">
+        <v>429</v>
+      </c>
+      <c r="E51" t="s">
         <v>430</v>
-      </c>
-      <c r="E51" t="s">
-        <v>431</v>
       </c>
       <c r="F51">
         <v>256</v>
@@ -7024,13 +7044,13 @@
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>432</v>
+      </c>
+      <c r="C52" t="s">
         <v>433</v>
       </c>
-      <c r="C52" t="s">
-        <v>434</v>
-      </c>
       <c r="E52" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="F52">
         <v>256</v>
@@ -7060,13 +7080,13 @@
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>434</v>
+      </c>
+      <c r="C53" t="s">
         <v>435</v>
       </c>
-      <c r="C53" t="s">
-        <v>436</v>
-      </c>
       <c r="E53" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="F53">
         <v>256</v>
@@ -7096,13 +7116,13 @@
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>436</v>
+      </c>
+      <c r="C54" t="s">
         <v>437</v>
       </c>
-      <c r="C54" t="s">
-        <v>438</v>
-      </c>
       <c r="E54" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="F54">
         <v>256</v>
@@ -7132,13 +7152,13 @@
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>438</v>
+      </c>
+      <c r="C55" t="s">
         <v>439</v>
       </c>
-      <c r="C55" t="s">
-        <v>440</v>
-      </c>
       <c r="E55" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="F55">
         <v>256</v>
@@ -7168,13 +7188,13 @@
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C56" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="E56" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="F56">
         <v>256</v>
@@ -7204,13 +7224,13 @@
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>441</v>
+      </c>
+      <c r="C57" t="s">
         <v>442</v>
       </c>
-      <c r="C57" t="s">
-        <v>443</v>
-      </c>
       <c r="E57" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="F57">
         <v>256</v>

</xml_diff>